<commit_message>
Re-specify RoBMA meta-regression under treatment contrasts; tighten Section 9-10 prose
Re-run Table 10, Table 10 FYI, and Table 12 under RoBMA's treatment-coding + pooled_effect() convention (per correspondence with the package author), superseding the earlier mean-difference/marginal_means() results. Reconciled Appendix C and the Section 9/10 narrative to match. Also trimmed redundant historical framing and correspondence narration from Sections 9.6 and 10 for a cleaner read.
</commit_message>
<xml_diff>
--- a/Table10_FYI_RoBMA.xlsx
+++ b/Table10_FYI_RoBMA.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">Component</t>
   </si>
@@ -37,15 +37,12 @@
     <t xml:space="preserve">Effect</t>
   </si>
   <si>
-    <t xml:space="preserve">0.440904888269833</t>
+    <t xml:space="preserve">119999</t>
   </si>
   <si>
     <t xml:space="preserve">Heterogeneity</t>
   </si>
   <si>
-    <t xml:space="preserve">119999</t>
-  </si>
-  <si>
     <t xml:space="preserve">Publication Bias</t>
   </si>
   <si>
@@ -97,28 +94,16 @@
     <t xml:space="preserve">intercept</t>
   </si>
   <si>
-    <t xml:space="preserve">Endog_FE[dif: 0]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endog_FE[dif: 1]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endog_IV[dif: 0]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endog_IV[dif: 1]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaggedDV[dif: 0]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaggedDV[dif: 1]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg_OECDEurope[dif: 0]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg_OECDEurope[dif: 1]</t>
+    <t xml:space="preserve">Endog_FE[1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endog_IV[1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LaggedDV[1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_OECDEurope[1]</t>
   </si>
   <si>
     <t xml:space="preserve">tau</t>
@@ -514,14 +499,12 @@
         <v>0.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.305991666666667</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="n">
-        <v>7.54005683227861</v>
-      </c>
+      <c r="E2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -534,13 +517,13 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="n">
         <v>0.5</v>
@@ -549,7 +532,7 @@
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E4"/>
     </row>
@@ -566,7 +549,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -583,70 +566,70 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
         <v>0.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.952733333333333</v>
+        <v>0.931041666666667</v>
       </c>
       <c r="D2" t="n">
-        <v>20.1565585331453</v>
+        <v>13.5015105740181</v>
       </c>
       <c r="E2" t="n">
-        <v>11.0211503865097</v>
+        <v>3.12458801739193</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="n">
         <v>0.5</v>
       </c>
       <c r="C3" t="n">
-        <v>0.230633333333333</v>
+        <v>0.291408333333333</v>
       </c>
       <c r="D3" t="n">
-        <v>0.299770373900611</v>
+        <v>0.411250014700521</v>
       </c>
       <c r="E3" t="n">
-        <v>4.42971334743952</v>
+        <v>1.28832718758186</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="n">
         <v>0.5</v>
       </c>
       <c r="C4" t="n">
-        <v>0.725066666666667</v>
+        <v>0.482033333333333</v>
       </c>
       <c r="D4" t="n">
-        <v>2.6372453928225</v>
+        <v>0.930626166419975</v>
       </c>
       <c r="E4" t="n">
-        <v>10.4371940991071</v>
+        <v>1.10942549992903</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="n">
         <v>0.5</v>
       </c>
       <c r="C5" t="n">
-        <v>0.183633333333333</v>
+        <v>0.22165</v>
       </c>
       <c r="D5" t="n">
-        <v>0.224939773794455</v>
+        <v>0.284769062760969</v>
       </c>
       <c r="E5" t="n">
-        <v>5.96859804632424</v>
+        <v>1.93121441776297</v>
       </c>
     </row>
   </sheetData>
@@ -662,322 +645,194 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>23</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0225101387273841</v>
+        <v>0.140669554310329</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0400630404523075</v>
+        <v>0.0273188541174808</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.0883415698680727</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.140241006875106</v>
       </c>
       <c r="F2" t="n">
-        <v>0.124981514250525</v>
+        <v>0.19595649201228</v>
       </c>
       <c r="G2" t="n">
-        <v>0.00162675063920968</v>
+        <v>0.000239456608278984</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0406047723997937</v>
+        <v>0.00876525081356764</v>
       </c>
       <c r="I2" t="n">
-        <v>624.020803568599</v>
+        <v>13028.9375322662</v>
       </c>
       <c r="J2" t="n">
-        <v>1.00423305336375</v>
+        <v>1.00013537748336</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0526846244574811</v>
+        <v>-0.0896276451902364</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0192630084961855</v>
+        <v>0.0390197692371208</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>-0.157330740937893</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0545940394711193</v>
+        <v>-0.0932558927327807</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0849532290183281</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.000374127712695685</v>
+        <v>0.000243837892609345</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0194220810715922</v>
+        <v>0.00624908597299888</v>
       </c>
       <c r="I3" t="n">
-        <v>2741.95953283013</v>
+        <v>25650.0284717649</v>
       </c>
       <c r="J3" t="n">
-        <v>1.0008936658702</v>
+        <v>1.00004276920644</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0526846244574811</v>
+        <v>-0.0129878387250401</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0192630084961855</v>
+        <v>0.025176210789618</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.0849532290183281</v>
+        <v>-0.0824007831271142</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.0545940394711193</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.000374127712695685</v>
+        <v>0.000157226919966034</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0194220810715922</v>
+        <v>0.00624505892804451</v>
       </c>
       <c r="I4" t="n">
-        <v>2741.95953283013</v>
+        <v>25662.1784785901</v>
       </c>
       <c r="J4" t="n">
-        <v>1.0008936658702</v>
+        <v>1.00018805807946</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0060142889021589</v>
+        <v>-0.0417661024435687</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0129876887025952</v>
+        <v>0.0552022257206233</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>-0.166278060478271</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.044217525440268</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.000349132573393306</v>
+        <v>0.000334007638412452</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0268818094880533</v>
+        <v>0.0060506190475517</v>
       </c>
       <c r="I5" t="n">
-        <v>1452.30819789641</v>
+        <v>27323.9191495843</v>
       </c>
       <c r="J5" t="n">
-        <v>1.00681021764997</v>
+        <v>1.00012697171002</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.0060142889021589</v>
+        <v>-0.00944030323143235</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0129876887025952</v>
+        <v>0.0260650206496691</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.044217525440268</v>
+        <v>-0.0916288888940527</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>0.00612842804901542</v>
       </c>
       <c r="G6" t="n">
-        <v>0.000349132573393306</v>
+        <v>0.000257733206780889</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0268818094880533</v>
+        <v>0.00988808757318829</v>
       </c>
       <c r="I6" t="n">
-        <v>1452.30819789641</v>
+        <v>10264.9908630016</v>
       </c>
       <c r="J6" t="n">
-        <v>1.00681021764997</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.0443445240309221</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.0328531738432523</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.0519247651530759</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.0973299259107073</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.00186674804065823</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0568209345485092</v>
-      </c>
-      <c r="I7" t="n">
-        <v>491.929125603847</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.00209582870187</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>31</v>
-      </c>
-      <c r="B8" t="n">
-        <v>-0.0443445240309221</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.0328531738432523</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.0973299259107073</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-0.0519247651530759</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.00186674804065823</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0568209345485092</v>
-      </c>
-      <c r="I8" t="n">
-        <v>491.929125603847</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.00209582870187</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.00518200241326859</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.0135657770621804</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.0491093922869115</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.00052321172823793</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.0385685040996711</v>
-      </c>
-      <c r="I9" t="n">
-        <v>930.647561755503</v>
-      </c>
-      <c r="J9" t="n">
-        <v>1.02386402820782</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" t="n">
-        <v>-0.00518200241326859</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.0135657770621804</v>
-      </c>
-      <c r="D10" t="n">
-        <v>-0.0491093922869115</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.00052321172823793</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.0385685040996711</v>
-      </c>
-      <c r="I10" t="n">
-        <v>930.647561755503</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.02386402820782</v>
+        <v>1.00015554162653</v>
       </c>
     </row>
   </sheetData>
@@ -993,98 +848,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>23</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B2" t="n">
-        <v>0.23773782795998</v>
+        <v>0.237934538772145</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0160096324466326</v>
+        <v>0.0160278121796058</v>
       </c>
       <c r="D2" t="n">
-        <v>0.210057806564577</v>
+        <v>0.21012018050579</v>
       </c>
       <c r="E2" t="n">
-        <v>0.236454877003323</v>
+        <v>0.236678889701582</v>
       </c>
       <c r="F2" t="n">
-        <v>0.272678708925671</v>
+        <v>0.27265572391983</v>
       </c>
       <c r="G2" t="n">
-        <v>0.000119589003901771</v>
+        <v>0.000118504271462922</v>
       </c>
       <c r="H2" t="n">
-        <v>0.00746981570628903</v>
+        <v>0.00739366484551832</v>
       </c>
       <c r="I2" t="n">
-        <v>17940.3763982235</v>
+        <v>18300.6263951543</v>
       </c>
       <c r="J2" t="n">
-        <v>1.00016241839989</v>
+        <v>1.00003583398932</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B3" t="n">
-        <v>0.535232348395844</v>
+        <v>0.540689996242606</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0612340762257274</v>
+        <v>0.0603067576257769</v>
       </c>
       <c r="D3" t="n">
-        <v>0.414108321757935</v>
+        <v>0.421960242880605</v>
       </c>
       <c r="E3" t="n">
-        <v>0.535628100399254</v>
+        <v>0.541144188898539</v>
       </c>
       <c r="F3" t="n">
-        <v>0.653157053492257</v>
+        <v>0.65695760935133</v>
       </c>
       <c r="G3" t="n">
-        <v>0.000462047133522161</v>
+        <v>0.000453980209755017</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00754558837172484</v>
+        <v>0.00752784974068928</v>
       </c>
       <c r="I3" t="n">
-        <v>17576.8847317488</v>
+        <v>17647.1629092138</v>
       </c>
       <c r="J3" t="n">
-        <v>1.00012252933255</v>
+        <v>1.00002757213313</v>
       </c>
     </row>
   </sheetData>
@@ -1100,39 +955,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>18</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>23</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -1156,16 +1011,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B3" t="n">
-        <v>0.991674753501118</v>
+        <v>0.991882536911987</v>
       </c>
       <c r="C3" t="n">
-        <v>0.026698029846074</v>
+        <v>0.0262460538453512</v>
       </c>
       <c r="D3" t="n">
-        <v>0.902289910420914</v>
+        <v>0.904507235416281</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -1174,149 +1029,149 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>0.000215610286708112</v>
+        <v>0.000208914592162806</v>
       </c>
       <c r="H3" t="n">
-        <v>0.00807588754493127</v>
+        <v>0.0079598477315404</v>
       </c>
       <c r="I3" t="n">
-        <v>15346.9418523985</v>
+        <v>15825.0899179575</v>
       </c>
       <c r="J3" t="n">
-        <v>1.00011419318571</v>
+        <v>1.00027284796921</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B4" t="n">
-        <v>0.690758842026082</v>
+        <v>0.703330652299298</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0727234905688459</v>
+        <v>0.0738771407802359</v>
       </c>
       <c r="D4" t="n">
-        <v>0.558688087483099</v>
+        <v>0.568902337528173</v>
       </c>
       <c r="E4" t="n">
-        <v>0.687395633455428</v>
+        <v>0.69966706650778</v>
       </c>
       <c r="F4" t="n">
-        <v>0.843661881840265</v>
+        <v>0.8584820786532</v>
       </c>
       <c r="G4" t="n">
-        <v>0.000361820785502322</v>
+        <v>0.000259990596600779</v>
       </c>
       <c r="H4" t="n">
-        <v>0.00497529453924922</v>
+        <v>0.00351922927518512</v>
       </c>
       <c r="I4" t="n">
-        <v>40425.0685339088</v>
+        <v>80885.240783042</v>
       </c>
       <c r="J4" t="n">
-        <v>1.00008915727764</v>
+        <v>1.00000631541142</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B5" t="n">
-        <v>0.224426152327369</v>
+        <v>0.235712460200444</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0385862919673724</v>
+        <v>0.0404508298944722</v>
       </c>
       <c r="D5" t="n">
-        <v>0.157967899987529</v>
+        <v>0.165667533074368</v>
       </c>
       <c r="E5" t="n">
-        <v>0.221291814289931</v>
+        <v>0.232618066903924</v>
       </c>
       <c r="F5" t="n">
-        <v>0.30873576307964</v>
+        <v>0.324176956285097</v>
       </c>
       <c r="G5" t="n">
-        <v>0.000290659659007524</v>
+        <v>0.00014510742714209</v>
       </c>
       <c r="H5" t="n">
-        <v>0.00753271807649458</v>
+        <v>0.00358725463780707</v>
       </c>
       <c r="I5" t="n">
-        <v>18414.4647547706</v>
+        <v>77714.3771433155</v>
       </c>
       <c r="J5" t="n">
-        <v>1.0001699202784</v>
+        <v>0.999995396010488</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B6" t="n">
-        <v>0.224426152327369</v>
+        <v>0.235712460200444</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0385862919673724</v>
+        <v>0.0404508298944722</v>
       </c>
       <c r="D6" t="n">
-        <v>0.157967899987529</v>
+        <v>0.165667533074368</v>
       </c>
       <c r="E6" t="n">
-        <v>0.221291814289931</v>
+        <v>0.232618066903924</v>
       </c>
       <c r="F6" t="n">
-        <v>0.30873576307964</v>
+        <v>0.324176956285097</v>
       </c>
       <c r="G6" t="n">
-        <v>0.000290659659007524</v>
+        <v>0.00014510742714209</v>
       </c>
       <c r="H6" t="n">
-        <v>0.00753271807649458</v>
+        <v>0.00358725463780707</v>
       </c>
       <c r="I6" t="n">
-        <v>18414.4647547706</v>
+        <v>77714.3771433155</v>
       </c>
       <c r="J6" t="n">
-        <v>1.0001699202784</v>
+        <v>0.999995396010488</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B7" t="n">
-        <v>0.224426152327369</v>
+        <v>0.235712460200444</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0385862919673724</v>
+        <v>0.0404508298944722</v>
       </c>
       <c r="D7" t="n">
-        <v>0.157967899987529</v>
+        <v>0.165667533074368</v>
       </c>
       <c r="E7" t="n">
-        <v>0.221291814289931</v>
+        <v>0.232618066903924</v>
       </c>
       <c r="F7" t="n">
-        <v>0.30873576307964</v>
+        <v>0.324176956285097</v>
       </c>
       <c r="G7" t="n">
-        <v>0.000290659659007524</v>
+        <v>0.00014510742714209</v>
       </c>
       <c r="H7" t="n">
-        <v>0.00753271807649458</v>
+        <v>0.00358725463780707</v>
       </c>
       <c r="I7" t="n">
-        <v>18414.4647547706</v>
+        <v>77714.3771433155</v>
       </c>
       <c r="J7" t="n">
-        <v>1.0001699202784</v>
+        <v>0.999995396010488</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
@@ -1344,7 +1199,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -1383,30 +1238,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0225101387273841</v>
+        <v>0.123480433848865</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.0754124579101622</v>
       </c>
       <c r="D2" t="n">
-        <v>0.124981514250525</v>
+        <v>0.172326889711699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>